<commit_message>
fix(dragon-gate): switch AI coach API to unified GAS proxy endpoint for 4 composition units
- Update dragon-gate/g8a-story-taipei-expansion.html
- Update dragon-gate/g7b-daan-park-flower-trip.html
- Update dragon-gate/g8b-hometown-flavor.html
- Update dragon-gate/g8b-news-discussion.html
- Remove direct Google API endpoint and empty apiKey setting
- Use unified GAS proxy endpoint with text/plain headers and response parsing
- Provide friendly connection error messages and diagnostic guidance
- Update 2026_CAP-Chinese catalog
</commit_message>
<xml_diff>
--- a/2026_CAP-Chinese目錄.xlsx
+++ b/2026_CAP-Chinese目錄.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\2026_CAP-Chinese\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{653DA5CC-5D78-4DEC-8DE5-F9627E36E10C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15AB93E-CF4E-4794-A923-C4298E980410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="11700" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="全站網頁連結目錄總表" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="1065">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1839" uniqueCount="1074">
   <si>
     <t>🏛️ 邁向會考之路——國文攻略 全站網頁資源目錄總表</t>
   </si>
@@ -3249,12 +3249,48 @@
     <t>(橘子)11-1[字音]常誤讀字-01成語類別</t>
     <phoneticPr fontId="8" type="noConversion"/>
   </si>
+  <si>
+    <t>https://oaoadna-1313.github.io/2026_CAP-Chinese/yuwen-practice/yuwen-interchangeable-chars.html</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]《三國演義》相關歇後語</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]《論語》相關佳句</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]生活常用詞</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集]方位詞判斷練習神器</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]《孟子》相關成語</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]四字以上成語(下)</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]《三國演義》相關成語</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>[語文學習集練習神器]《戰國策》與先秦歷史相關成語</t>
+    <phoneticPr fontId="8" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3349,6 +3385,14 @@
       <color rgb="FF0F172A"/>
       <name val="Segoe UI Emoji"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="新細明體"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="16">
@@ -3467,10 +3511,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3505,13 +3550,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3535,9 +3573,18 @@
     <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="超連結" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -3848,24 +3895,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
     </row>
     <row r="3" spans="1:6" ht="8" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.3">
@@ -9428,15 +9475,15 @@
   <dimension ref="A1:B258"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="51.8984375" customWidth="1"/>
-    <col min="2" max="2" width="53.59765625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="75.59765625" customWidth="1"/>
+    <col min="2" max="2" width="53.59765625" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="14" t="s">
         <v>31</v>
       </c>
     </row>
@@ -9444,7 +9491,7 @@
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="14" t="s">
         <v>35</v>
       </c>
     </row>
@@ -9452,7 +9499,7 @@
       <c r="A3" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="14" t="s">
         <v>39</v>
       </c>
     </row>
@@ -9460,23 +9507,23 @@
       <c r="A4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="17" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="17" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>51</v>
       </c>
     </row>
@@ -9484,7 +9531,7 @@
       <c r="A7" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="14" t="s">
         <v>55</v>
       </c>
     </row>
@@ -9492,7 +9539,7 @@
       <c r="A8" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="14" t="s">
         <v>59</v>
       </c>
     </row>
@@ -9500,7 +9547,7 @@
       <c r="A9" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>63</v>
       </c>
     </row>
@@ -9508,7 +9555,7 @@
       <c r="A10" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="14" t="s">
         <v>67</v>
       </c>
     </row>
@@ -9516,7 +9563,7 @@
       <c r="A11" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="14" t="s">
         <v>71</v>
       </c>
     </row>
@@ -9524,7 +9571,7 @@
       <c r="A12" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="14" t="s">
         <v>75</v>
       </c>
     </row>
@@ -9532,7 +9579,7 @@
       <c r="A13" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="14" t="s">
         <v>79</v>
       </c>
     </row>
@@ -9540,7 +9587,7 @@
       <c r="A14" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="14" t="s">
         <v>83</v>
       </c>
     </row>
@@ -9548,7 +9595,7 @@
       <c r="A15" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="14" t="s">
         <v>87</v>
       </c>
     </row>
@@ -9556,7 +9603,7 @@
       <c r="A16" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="14" t="s">
         <v>91</v>
       </c>
     </row>
@@ -9564,7 +9611,7 @@
       <c r="A17" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="14" t="s">
         <v>1058</v>
       </c>
     </row>
@@ -9572,7 +9619,7 @@
       <c r="A18" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="14" t="s">
         <v>99</v>
       </c>
     </row>
@@ -9580,7 +9627,7 @@
       <c r="A19" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>103</v>
       </c>
     </row>
@@ -9588,7 +9635,7 @@
       <c r="A20" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="14" t="s">
         <v>107</v>
       </c>
     </row>
@@ -9596,7 +9643,7 @@
       <c r="A21" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>111</v>
       </c>
     </row>
@@ -9604,7 +9651,7 @@
       <c r="A22" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="14" t="s">
         <v>115</v>
       </c>
     </row>
@@ -9612,7 +9659,7 @@
       <c r="A23" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="14" t="s">
         <v>119</v>
       </c>
     </row>
@@ -9620,7 +9667,7 @@
       <c r="A24" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="14" t="s">
         <v>123</v>
       </c>
     </row>
@@ -9628,7 +9675,7 @@
       <c r="A25" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="14" t="s">
         <v>127</v>
       </c>
     </row>
@@ -9636,23 +9683,23 @@
       <c r="A26" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="14" t="s">
         <v>1059</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="B27" s="17" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B27" s="14" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B28" s="17" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B28" s="14" t="s">
         <v>139</v>
       </c>
     </row>
@@ -9660,7 +9707,7 @@
       <c r="A29" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="14" t="s">
         <v>143</v>
       </c>
     </row>
@@ -9668,7 +9715,7 @@
       <c r="A30" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="14" t="s">
         <v>147</v>
       </c>
     </row>
@@ -9676,7 +9723,7 @@
       <c r="A31" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="14" t="s">
         <v>151</v>
       </c>
     </row>
@@ -9684,7 +9731,7 @@
       <c r="A32" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="14" t="s">
         <v>155</v>
       </c>
     </row>
@@ -9692,7 +9739,7 @@
       <c r="A33" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="14" t="s">
         <v>159</v>
       </c>
     </row>
@@ -9700,7 +9747,7 @@
       <c r="A34" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="14" t="s">
         <v>163</v>
       </c>
     </row>
@@ -9708,7 +9755,7 @@
       <c r="A35" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="14" t="s">
         <v>167</v>
       </c>
     </row>
@@ -9716,7 +9763,7 @@
       <c r="A36" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B36" s="14" t="s">
         <v>171</v>
       </c>
     </row>
@@ -9724,7 +9771,7 @@
       <c r="A37" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="14" t="s">
         <v>174</v>
       </c>
     </row>
@@ -9732,15 +9779,15 @@
       <c r="A38" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B38" s="14" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="B39" s="17" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B39" s="14" t="s">
         <v>182</v>
       </c>
     </row>
@@ -9748,7 +9795,7 @@
       <c r="A40" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="14" t="s">
         <v>186</v>
       </c>
     </row>
@@ -9756,15 +9803,15 @@
       <c r="A41" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="14" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="B42" s="17" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B42" s="14" t="s">
         <v>194</v>
       </c>
     </row>
@@ -9772,7 +9819,7 @@
       <c r="A43" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B43" s="14" t="s">
         <v>198</v>
       </c>
     </row>
@@ -9780,7 +9827,7 @@
       <c r="A44" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="B44" s="17" t="s">
+      <c r="B44" s="14" t="s">
         <v>202</v>
       </c>
     </row>
@@ -9788,7 +9835,7 @@
       <c r="A45" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B45" s="14" t="s">
         <v>206</v>
       </c>
     </row>
@@ -9796,7 +9843,7 @@
       <c r="A46" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B46" s="14" t="s">
         <v>210</v>
       </c>
     </row>
@@ -9804,7 +9851,7 @@
       <c r="A47" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="14" t="s">
         <v>214</v>
       </c>
     </row>
@@ -9812,7 +9859,7 @@
       <c r="A48" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="14" t="s">
         <v>218</v>
       </c>
     </row>
@@ -9820,7 +9867,7 @@
       <c r="A49" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="14" t="s">
         <v>222</v>
       </c>
     </row>
@@ -9828,7 +9875,7 @@
       <c r="A50" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="B50" s="17" t="s">
+      <c r="B50" s="14" t="s">
         <v>226</v>
       </c>
     </row>
@@ -9836,23 +9883,23 @@
       <c r="A51" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B51" s="14" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B52" s="17" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B52" s="14" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="B53" s="17" t="s">
+        <v>1073</v>
+      </c>
+      <c r="B53" s="14" t="s">
         <v>238</v>
       </c>
     </row>
@@ -9860,7 +9907,7 @@
       <c r="A54" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="B54" s="17" t="s">
+      <c r="B54" s="14" t="s">
         <v>242</v>
       </c>
     </row>
@@ -9868,7 +9915,7 @@
       <c r="A55" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B55" s="17" t="s">
+      <c r="B55" s="14" t="s">
         <v>246</v>
       </c>
     </row>
@@ -9876,7 +9923,7 @@
       <c r="A56" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B56" s="14" t="s">
         <v>250</v>
       </c>
     </row>
@@ -9884,7 +9931,7 @@
       <c r="A57" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B57" s="14" t="s">
         <v>254</v>
       </c>
     </row>
@@ -9892,7 +9939,7 @@
       <c r="A58" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="B58" s="17" t="s">
+      <c r="B58" s="14" t="s">
         <v>258</v>
       </c>
     </row>
@@ -9900,15 +9947,15 @@
       <c r="A59" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="B59" s="17" t="s">
-        <v>262</v>
+      <c r="B59" s="26" t="s">
+        <v>1065</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="B60" s="17" t="s">
+      <c r="B60" s="14" t="s">
         <v>266</v>
       </c>
     </row>
@@ -9916,7 +9963,7 @@
       <c r="A61" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="14" t="s">
         <v>270</v>
       </c>
     </row>
@@ -9924,7 +9971,7 @@
       <c r="A62" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="B62" s="17" t="s">
+      <c r="B62" s="14" t="s">
         <v>274</v>
       </c>
     </row>
@@ -9932,7 +9979,7 @@
       <c r="A63" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B63" s="17" t="s">
+      <c r="B63" s="14" t="s">
         <v>278</v>
       </c>
     </row>
@@ -9940,7 +9987,7 @@
       <c r="A64" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="B64" s="17" t="s">
+      <c r="B64" s="14" t="s">
         <v>282</v>
       </c>
     </row>
@@ -9948,7 +9995,7 @@
       <c r="A65" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="B65" s="17" t="s">
+      <c r="B65" s="14" t="s">
         <v>286</v>
       </c>
     </row>
@@ -9956,7 +10003,7 @@
       <c r="A66" s="4" t="s">
         <v>287</v>
       </c>
-      <c r="B66" s="17" t="s">
+      <c r="B66" s="14" t="s">
         <v>290</v>
       </c>
     </row>
@@ -9964,7 +10011,7 @@
       <c r="A67" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="14" t="s">
         <v>294</v>
       </c>
     </row>
@@ -9972,7 +10019,7 @@
       <c r="A68" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="B68" s="17" t="s">
+      <c r="B68" s="14" t="s">
         <v>298</v>
       </c>
     </row>
@@ -9980,7 +10027,7 @@
       <c r="A69" s="9" t="s">
         <v>299</v>
       </c>
-      <c r="B69" s="17" t="s">
+      <c r="B69" s="14" t="s">
         <v>302</v>
       </c>
     </row>
@@ -9988,7 +10035,7 @@
       <c r="A70" s="4" t="s">
         <v>303</v>
       </c>
-      <c r="B70" s="17" t="s">
+      <c r="B70" s="14" t="s">
         <v>306</v>
       </c>
     </row>
@@ -9996,7 +10043,7 @@
       <c r="A71" s="9" t="s">
         <v>307</v>
       </c>
-      <c r="B71" s="17" t="s">
+      <c r="B71" s="14" t="s">
         <v>310</v>
       </c>
     </row>
@@ -10004,7 +10051,7 @@
       <c r="A72" s="4" t="s">
         <v>239</v>
       </c>
-      <c r="B72" s="17" t="s">
+      <c r="B72" s="14" t="s">
         <v>313</v>
       </c>
     </row>
@@ -10012,7 +10059,7 @@
       <c r="A73" s="9" t="s">
         <v>314</v>
       </c>
-      <c r="B73" s="17" t="s">
+      <c r="B73" s="14" t="s">
         <v>317</v>
       </c>
     </row>
@@ -10020,7 +10067,7 @@
       <c r="A74" s="4" t="s">
         <v>318</v>
       </c>
-      <c r="B74" s="17" t="s">
+      <c r="B74" s="14" t="s">
         <v>321</v>
       </c>
     </row>
@@ -10028,7 +10075,7 @@
       <c r="A75" s="9" t="s">
         <v>322</v>
       </c>
-      <c r="B75" s="17" t="s">
+      <c r="B75" s="14" t="s">
         <v>325</v>
       </c>
     </row>
@@ -10036,7 +10083,7 @@
       <c r="A76" s="4" t="s">
         <v>326</v>
       </c>
-      <c r="B76" s="17" t="s">
+      <c r="B76" s="14" t="s">
         <v>329</v>
       </c>
     </row>
@@ -10044,7 +10091,7 @@
       <c r="A77" s="9" t="s">
         <v>330</v>
       </c>
-      <c r="B77" s="17" t="s">
+      <c r="B77" s="14" t="s">
         <v>333</v>
       </c>
     </row>
@@ -10052,7 +10099,7 @@
       <c r="A78" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="B78" s="17" t="s">
+      <c r="B78" s="14" t="s">
         <v>337</v>
       </c>
     </row>
@@ -10060,7 +10107,7 @@
       <c r="A79" s="9" t="s">
         <v>338</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B79" s="14" t="s">
         <v>341</v>
       </c>
     </row>
@@ -10068,7 +10115,7 @@
       <c r="A80" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="B80" s="17" t="s">
+      <c r="B80" s="14" t="s">
         <v>345</v>
       </c>
     </row>
@@ -10076,7 +10123,7 @@
       <c r="A81" s="9" t="s">
         <v>346</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B81" s="14" t="s">
         <v>349</v>
       </c>
     </row>
@@ -10084,7 +10131,7 @@
       <c r="A82" s="4" t="s">
         <v>350</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B82" s="14" t="s">
         <v>353</v>
       </c>
     </row>
@@ -10092,7 +10139,7 @@
       <c r="A83" s="9" t="s">
         <v>354</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B83" s="14" t="s">
         <v>357</v>
       </c>
     </row>
@@ -10100,7 +10147,7 @@
       <c r="A84" s="4" t="s">
         <v>358</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B84" s="14" t="s">
         <v>361</v>
       </c>
     </row>
@@ -10108,7 +10155,7 @@
       <c r="A85" s="9" t="s">
         <v>362</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B85" s="14" t="s">
         <v>365</v>
       </c>
     </row>
@@ -10116,7 +10163,7 @@
       <c r="A86" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B86" s="14" t="s">
         <v>369</v>
       </c>
     </row>
@@ -10124,7 +10171,7 @@
       <c r="A87" s="9" t="s">
         <v>370</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B87" s="14" t="s">
         <v>373</v>
       </c>
     </row>
@@ -10132,7 +10179,7 @@
       <c r="A88" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B88" s="14" t="s">
         <v>377</v>
       </c>
     </row>
@@ -10140,7 +10187,7 @@
       <c r="A89" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B89" s="14" t="s">
         <v>381</v>
       </c>
     </row>
@@ -10148,7 +10195,7 @@
       <c r="A90" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B90" s="14" t="s">
         <v>385</v>
       </c>
     </row>
@@ -10156,7 +10203,7 @@
       <c r="A91" s="9" t="s">
         <v>386</v>
       </c>
-      <c r="B91" s="17" t="s">
+      <c r="B91" s="14" t="s">
         <v>389</v>
       </c>
     </row>
@@ -10164,7 +10211,7 @@
       <c r="A92" s="4" t="s">
         <v>390</v>
       </c>
-      <c r="B92" s="17" t="s">
+      <c r="B92" s="14" t="s">
         <v>393</v>
       </c>
     </row>
@@ -10172,7 +10219,7 @@
       <c r="A93" s="9" t="s">
         <v>394</v>
       </c>
-      <c r="B93" s="17" t="s">
+      <c r="B93" s="14" t="s">
         <v>397</v>
       </c>
     </row>
@@ -10180,7 +10227,7 @@
       <c r="A94" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="B94" s="17" t="s">
+      <c r="B94" s="14" t="s">
         <v>401</v>
       </c>
     </row>
@@ -10188,7 +10235,7 @@
       <c r="A95" s="9" t="s">
         <v>402</v>
       </c>
-      <c r="B95" s="17" t="s">
+      <c r="B95" s="14" t="s">
         <v>405</v>
       </c>
     </row>
@@ -10196,7 +10243,7 @@
       <c r="A96" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="B96" s="17" t="s">
+      <c r="B96" s="14" t="s">
         <v>409</v>
       </c>
     </row>
@@ -10204,7 +10251,7 @@
       <c r="A97" s="9" t="s">
         <v>410</v>
       </c>
-      <c r="B97" s="17" t="s">
+      <c r="B97" s="14" t="s">
         <v>413</v>
       </c>
     </row>
@@ -10212,7 +10259,7 @@
       <c r="A98" s="4" t="s">
         <v>414</v>
       </c>
-      <c r="B98" s="17" t="s">
+      <c r="B98" s="14" t="s">
         <v>417</v>
       </c>
     </row>
@@ -10220,7 +10267,7 @@
       <c r="A99" s="9" t="s">
         <v>418</v>
       </c>
-      <c r="B99" s="17" t="s">
+      <c r="B99" s="14" t="s">
         <v>1060</v>
       </c>
     </row>
@@ -10228,7 +10275,7 @@
       <c r="A100" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="B100" s="17" t="s">
+      <c r="B100" s="14" t="s">
         <v>425</v>
       </c>
     </row>
@@ -10236,7 +10283,7 @@
       <c r="A101" s="9" t="s">
         <v>426</v>
       </c>
-      <c r="B101" s="17" t="s">
+      <c r="B101" s="14" t="s">
         <v>429</v>
       </c>
     </row>
@@ -10244,7 +10291,7 @@
       <c r="A102" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="B102" s="17" t="s">
+      <c r="B102" s="14" t="s">
         <v>433</v>
       </c>
     </row>
@@ -10252,7 +10299,7 @@
       <c r="A103" s="9" t="s">
         <v>434</v>
       </c>
-      <c r="B103" s="17" t="s">
+      <c r="B103" s="14" t="s">
         <v>437</v>
       </c>
     </row>
@@ -10260,7 +10307,7 @@
       <c r="A104" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="B104" s="17" t="s">
+      <c r="B104" s="14" t="s">
         <v>441</v>
       </c>
     </row>
@@ -10268,7 +10315,7 @@
       <c r="A105" s="9" t="s">
         <v>442</v>
       </c>
-      <c r="B105" s="17" t="s">
+      <c r="B105" s="14" t="s">
         <v>445</v>
       </c>
     </row>
@@ -10276,7 +10323,7 @@
       <c r="A106" s="4" t="s">
         <v>446</v>
       </c>
-      <c r="B106" s="17" t="s">
+      <c r="B106" s="14" t="s">
         <v>449</v>
       </c>
     </row>
@@ -10284,7 +10331,7 @@
       <c r="A107" s="9" t="s">
         <v>451</v>
       </c>
-      <c r="B107" s="17" t="s">
+      <c r="B107" s="14" t="s">
         <v>454</v>
       </c>
     </row>
@@ -10292,7 +10339,7 @@
       <c r="A108" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="B108" s="17" t="s">
+      <c r="B108" s="14" t="s">
         <v>458</v>
       </c>
     </row>
@@ -10300,7 +10347,7 @@
       <c r="A109" s="9" t="s">
         <v>459</v>
       </c>
-      <c r="B109" s="17" t="s">
+      <c r="B109" s="14" t="s">
         <v>462</v>
       </c>
     </row>
@@ -10308,7 +10355,7 @@
       <c r="A110" s="4" t="s">
         <v>463</v>
       </c>
-      <c r="B110" s="17" t="s">
+      <c r="B110" s="14" t="s">
         <v>466</v>
       </c>
     </row>
@@ -10316,7 +10363,7 @@
       <c r="A111" s="9" t="s">
         <v>467</v>
       </c>
-      <c r="B111" s="17" t="s">
+      <c r="B111" s="14" t="s">
         <v>470</v>
       </c>
     </row>
@@ -10324,7 +10371,7 @@
       <c r="A112" s="4" t="s">
         <v>471</v>
       </c>
-      <c r="B112" s="17" t="s">
+      <c r="B112" s="14" t="s">
         <v>474</v>
       </c>
     </row>
@@ -10332,7 +10379,7 @@
       <c r="A113" s="9" t="s">
         <v>475</v>
       </c>
-      <c r="B113" s="17" t="s">
+      <c r="B113" s="14" t="s">
         <v>478</v>
       </c>
     </row>
@@ -10340,7 +10387,7 @@
       <c r="A114" s="4" t="s">
         <v>479</v>
       </c>
-      <c r="B114" s="17" t="s">
+      <c r="B114" s="14" t="s">
         <v>482</v>
       </c>
     </row>
@@ -10348,7 +10395,7 @@
       <c r="A115" s="9" t="s">
         <v>483</v>
       </c>
-      <c r="B115" s="17" t="s">
+      <c r="B115" s="14" t="s">
         <v>486</v>
       </c>
     </row>
@@ -10356,7 +10403,7 @@
       <c r="A116" s="4" t="s">
         <v>487</v>
       </c>
-      <c r="B116" s="17" t="s">
+      <c r="B116" s="14" t="s">
         <v>490</v>
       </c>
     </row>
@@ -10364,7 +10411,7 @@
       <c r="A117" s="9" t="s">
         <v>1064</v>
       </c>
-      <c r="B117" s="17" t="s">
+      <c r="B117" s="14" t="s">
         <v>493</v>
       </c>
     </row>
@@ -10372,7 +10419,7 @@
       <c r="A118" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="B118" s="17" t="s">
+      <c r="B118" s="14" t="s">
         <v>497</v>
       </c>
     </row>
@@ -10380,7 +10427,7 @@
       <c r="A119" s="9" t="s">
         <v>498</v>
       </c>
-      <c r="B119" s="17" t="s">
+      <c r="B119" s="14" t="s">
         <v>501</v>
       </c>
     </row>
@@ -10388,7 +10435,7 @@
       <c r="A120" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="B120" s="17" t="s">
+      <c r="B120" s="14" t="s">
         <v>505</v>
       </c>
     </row>
@@ -10396,7 +10443,7 @@
       <c r="A121" s="9" t="s">
         <v>506</v>
       </c>
-      <c r="B121" s="17" t="s">
+      <c r="B121" s="14" t="s">
         <v>509</v>
       </c>
     </row>
@@ -10404,7 +10451,7 @@
       <c r="A122" s="4" t="s">
         <v>510</v>
       </c>
-      <c r="B122" s="17" t="s">
+      <c r="B122" s="14" t="s">
         <v>513</v>
       </c>
     </row>
@@ -10412,7 +10459,7 @@
       <c r="A123" s="9" t="s">
         <v>514</v>
       </c>
-      <c r="B123" s="17" t="s">
+      <c r="B123" s="14" t="s">
         <v>517</v>
       </c>
     </row>
@@ -10420,7 +10467,7 @@
       <c r="A124" s="4" t="s">
         <v>518</v>
       </c>
-      <c r="B124" s="17" t="s">
+      <c r="B124" s="14" t="s">
         <v>521</v>
       </c>
     </row>
@@ -10428,7 +10475,7 @@
       <c r="A125" s="9" t="s">
         <v>522</v>
       </c>
-      <c r="B125" s="17" t="s">
+      <c r="B125" s="14" t="s">
         <v>525</v>
       </c>
     </row>
@@ -10436,7 +10483,7 @@
       <c r="A126" s="4" t="s">
         <v>526</v>
       </c>
-      <c r="B126" s="17" t="s">
+      <c r="B126" s="14" t="s">
         <v>529</v>
       </c>
     </row>
@@ -10444,7 +10491,7 @@
       <c r="A127" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="B127" s="17" t="s">
+      <c r="B127" s="14" t="s">
         <v>533</v>
       </c>
     </row>
@@ -10452,7 +10499,7 @@
       <c r="A128" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="B128" s="17" t="s">
+      <c r="B128" s="14" t="s">
         <v>537</v>
       </c>
     </row>
@@ -10460,7 +10507,7 @@
       <c r="A129" s="9" t="s">
         <v>538</v>
       </c>
-      <c r="B129" s="17" t="s">
+      <c r="B129" s="14" t="s">
         <v>541</v>
       </c>
     </row>
@@ -10468,7 +10515,7 @@
       <c r="A130" s="4" t="s">
         <v>542</v>
       </c>
-      <c r="B130" s="17" t="s">
+      <c r="B130" s="14" t="s">
         <v>545</v>
       </c>
     </row>
@@ -10476,7 +10523,7 @@
       <c r="A131" s="9" t="s">
         <v>546</v>
       </c>
-      <c r="B131" s="17" t="s">
+      <c r="B131" s="14" t="s">
         <v>549</v>
       </c>
     </row>
@@ -10484,39 +10531,39 @@
       <c r="A132" s="4" t="s">
         <v>551</v>
       </c>
-      <c r="B132" s="18" t="s">
+      <c r="B132" s="15" t="s">
         <v>554</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A133" s="15" t="s">
+      <c r="A133" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B133" s="19" t="s">
+      <c r="B133" s="16" t="s">
         <v>557</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A134" s="16" t="s">
+      <c r="A134" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B134" s="19" t="s">
+      <c r="B134" s="16" t="s">
         <v>560</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A135" s="15" t="s">
+      <c r="A135" s="12" t="s">
         <v>382</v>
       </c>
-      <c r="B135" s="19" t="s">
+      <c r="B135" s="16" t="s">
         <v>563</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A136" s="16" t="s">
+      <c r="A136" s="13" t="s">
         <v>386</v>
       </c>
-      <c r="B136" s="19" t="s">
+      <c r="B136" s="16" t="s">
         <v>566</v>
       </c>
     </row>
@@ -10524,7 +10571,7 @@
       <c r="A137" s="9" t="s">
         <v>567</v>
       </c>
-      <c r="B137" s="18" t="s">
+      <c r="B137" s="15" t="s">
         <v>570</v>
       </c>
     </row>
@@ -10532,7 +10579,7 @@
       <c r="A138" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="B138" s="17" t="s">
+      <c r="B138" s="14" t="s">
         <v>573</v>
       </c>
     </row>
@@ -10540,7 +10587,7 @@
       <c r="A139" s="9" t="s">
         <v>575</v>
       </c>
-      <c r="B139" s="17" t="s">
+      <c r="B139" s="14" t="s">
         <v>578</v>
       </c>
     </row>
@@ -10548,7 +10595,7 @@
       <c r="A140" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="B140" s="17" t="s">
+      <c r="B140" s="14" t="s">
         <v>582</v>
       </c>
     </row>
@@ -10556,7 +10603,7 @@
       <c r="A141" s="9" t="s">
         <v>583</v>
       </c>
-      <c r="B141" s="17" t="s">
+      <c r="B141" s="14" t="s">
         <v>1061</v>
       </c>
     </row>
@@ -10564,7 +10611,7 @@
       <c r="A142" s="4" t="s">
         <v>587</v>
       </c>
-      <c r="B142" s="17" t="s">
+      <c r="B142" s="14" t="s">
         <v>590</v>
       </c>
     </row>
@@ -10572,7 +10619,7 @@
       <c r="A143" s="9" t="s">
         <v>591</v>
       </c>
-      <c r="B143" s="17" t="s">
+      <c r="B143" s="14" t="s">
         <v>594</v>
       </c>
     </row>
@@ -10580,7 +10627,7 @@
       <c r="A144" s="4" t="s">
         <v>595</v>
       </c>
-      <c r="B144" s="17" t="s">
+      <c r="B144" s="14" t="s">
         <v>598</v>
       </c>
     </row>
@@ -10588,7 +10635,7 @@
       <c r="A145" s="9" t="s">
         <v>599</v>
       </c>
-      <c r="B145" s="17" t="s">
+      <c r="B145" s="14" t="s">
         <v>602</v>
       </c>
     </row>
@@ -10596,7 +10643,7 @@
       <c r="A146" s="4" t="s">
         <v>603</v>
       </c>
-      <c r="B146" s="17" t="s">
+      <c r="B146" s="14" t="s">
         <v>606</v>
       </c>
     </row>
@@ -10604,7 +10651,7 @@
       <c r="A147" s="9" t="s">
         <v>607</v>
       </c>
-      <c r="B147" s="17" t="s">
+      <c r="B147" s="14" t="s">
         <v>610</v>
       </c>
     </row>
@@ -10612,7 +10659,7 @@
       <c r="A148" s="4" t="s">
         <v>611</v>
       </c>
-      <c r="B148" s="17" t="s">
+      <c r="B148" s="14" t="s">
         <v>614</v>
       </c>
     </row>
@@ -10620,7 +10667,7 @@
       <c r="A149" s="9" t="s">
         <v>615</v>
       </c>
-      <c r="B149" s="17" t="s">
+      <c r="B149" s="14" t="s">
         <v>618</v>
       </c>
     </row>
@@ -10628,7 +10675,7 @@
       <c r="A150" s="4" t="s">
         <v>619</v>
       </c>
-      <c r="B150" s="17" t="s">
+      <c r="B150" s="14" t="s">
         <v>1062</v>
       </c>
     </row>
@@ -10636,7 +10683,7 @@
       <c r="A151" s="9" t="s">
         <v>623</v>
       </c>
-      <c r="B151" s="17" t="s">
+      <c r="B151" s="14" t="s">
         <v>626</v>
       </c>
     </row>
@@ -10644,7 +10691,7 @@
       <c r="A152" s="4" t="s">
         <v>627</v>
       </c>
-      <c r="B152" s="17" t="s">
+      <c r="B152" s="14" t="s">
         <v>630</v>
       </c>
     </row>
@@ -10652,7 +10699,7 @@
       <c r="A153" s="9" t="s">
         <v>631</v>
       </c>
-      <c r="B153" s="17" t="s">
+      <c r="B153" s="14" t="s">
         <v>634</v>
       </c>
     </row>
@@ -10660,7 +10707,7 @@
       <c r="A154" s="4" t="s">
         <v>635</v>
       </c>
-      <c r="B154" s="17" t="s">
+      <c r="B154" s="14" t="s">
         <v>638</v>
       </c>
     </row>
@@ -10668,7 +10715,7 @@
       <c r="A155" s="9" t="s">
         <v>639</v>
       </c>
-      <c r="B155" s="17" t="s">
+      <c r="B155" s="14" t="s">
         <v>642</v>
       </c>
     </row>
@@ -10676,7 +10723,7 @@
       <c r="A156" s="4" t="s">
         <v>643</v>
       </c>
-      <c r="B156" s="17" t="s">
+      <c r="B156" s="14" t="s">
         <v>646</v>
       </c>
     </row>
@@ -10684,7 +10731,7 @@
       <c r="A157" s="9" t="s">
         <v>647</v>
       </c>
-      <c r="B157" s="17" t="s">
+      <c r="B157" s="14" t="s">
         <v>650</v>
       </c>
     </row>
@@ -10692,7 +10739,7 @@
       <c r="A158" s="4" t="s">
         <v>651</v>
       </c>
-      <c r="B158" s="17" t="s">
+      <c r="B158" s="14" t="s">
         <v>654</v>
       </c>
     </row>
@@ -10700,7 +10747,7 @@
       <c r="A159" s="9" t="s">
         <v>655</v>
       </c>
-      <c r="B159" s="17" t="s">
+      <c r="B159" s="14" t="s">
         <v>658</v>
       </c>
     </row>
@@ -10708,7 +10755,7 @@
       <c r="A160" s="4" t="s">
         <v>659</v>
       </c>
-      <c r="B160" s="17" t="s">
+      <c r="B160" s="14" t="s">
         <v>662</v>
       </c>
     </row>
@@ -10716,7 +10763,7 @@
       <c r="A161" s="9" t="s">
         <v>663</v>
       </c>
-      <c r="B161" s="17" t="s">
+      <c r="B161" s="14" t="s">
         <v>666</v>
       </c>
     </row>
@@ -10724,7 +10771,7 @@
       <c r="A162" s="4" t="s">
         <v>667</v>
       </c>
-      <c r="B162" s="17" t="s">
+      <c r="B162" s="14" t="s">
         <v>670</v>
       </c>
     </row>
@@ -10732,7 +10779,7 @@
       <c r="A163" s="9" t="s">
         <v>671</v>
       </c>
-      <c r="B163" s="17" t="s">
+      <c r="B163" s="14" t="s">
         <v>674</v>
       </c>
     </row>
@@ -10740,7 +10787,7 @@
       <c r="A164" s="4" t="s">
         <v>675</v>
       </c>
-      <c r="B164" s="17" t="s">
+      <c r="B164" s="14" t="s">
         <v>678</v>
       </c>
     </row>
@@ -10748,7 +10795,7 @@
       <c r="A165" s="9" t="s">
         <v>679</v>
       </c>
-      <c r="B165" s="17" t="s">
+      <c r="B165" s="14" t="s">
         <v>682</v>
       </c>
     </row>
@@ -10756,7 +10803,7 @@
       <c r="A166" s="4" t="s">
         <v>683</v>
       </c>
-      <c r="B166" s="17" t="s">
+      <c r="B166" s="14" t="s">
         <v>686</v>
       </c>
     </row>
@@ -10764,7 +10811,7 @@
       <c r="A167" s="9" t="s">
         <v>687</v>
       </c>
-      <c r="B167" s="17" t="s">
+      <c r="B167" s="14" t="s">
         <v>690</v>
       </c>
     </row>
@@ -10772,7 +10819,7 @@
       <c r="A168" s="4" t="s">
         <v>691</v>
       </c>
-      <c r="B168" s="17" t="s">
+      <c r="B168" s="14" t="s">
         <v>694</v>
       </c>
     </row>
@@ -10780,7 +10827,7 @@
       <c r="A169" s="9" t="s">
         <v>695</v>
       </c>
-      <c r="B169" s="17" t="s">
+      <c r="B169" s="14" t="s">
         <v>698</v>
       </c>
     </row>
@@ -10788,7 +10835,7 @@
       <c r="A170" s="4" t="s">
         <v>699</v>
       </c>
-      <c r="B170" s="17" t="s">
+      <c r="B170" s="14" t="s">
         <v>702</v>
       </c>
     </row>
@@ -10796,7 +10843,7 @@
       <c r="A171" s="9" t="s">
         <v>703</v>
       </c>
-      <c r="B171" s="17" t="s">
+      <c r="B171" s="14" t="s">
         <v>706</v>
       </c>
     </row>
@@ -10804,7 +10851,7 @@
       <c r="A172" s="4" t="s">
         <v>707</v>
       </c>
-      <c r="B172" s="17" t="s">
+      <c r="B172" s="14" t="s">
         <v>710</v>
       </c>
     </row>
@@ -10812,7 +10859,7 @@
       <c r="A173" s="9" t="s">
         <v>711</v>
       </c>
-      <c r="B173" s="17" t="s">
+      <c r="B173" s="14" t="s">
         <v>714</v>
       </c>
     </row>
@@ -10820,7 +10867,7 @@
       <c r="A174" s="4" t="s">
         <v>715</v>
       </c>
-      <c r="B174" s="17" t="s">
+      <c r="B174" s="14" t="s">
         <v>718</v>
       </c>
     </row>
@@ -10828,7 +10875,7 @@
       <c r="A175" s="9" t="s">
         <v>719</v>
       </c>
-      <c r="B175" s="17" t="s">
+      <c r="B175" s="14" t="s">
         <v>722</v>
       </c>
     </row>
@@ -10836,7 +10883,7 @@
       <c r="A176" s="4" t="s">
         <v>723</v>
       </c>
-      <c r="B176" s="17" t="s">
+      <c r="B176" s="14" t="s">
         <v>726</v>
       </c>
     </row>
@@ -10844,7 +10891,7 @@
       <c r="A177" s="9" t="s">
         <v>727</v>
       </c>
-      <c r="B177" s="17" t="s">
+      <c r="B177" s="14" t="s">
         <v>730</v>
       </c>
     </row>
@@ -10852,7 +10899,7 @@
       <c r="A178" s="4" t="s">
         <v>731</v>
       </c>
-      <c r="B178" s="17" t="s">
+      <c r="B178" s="14" t="s">
         <v>734</v>
       </c>
     </row>
@@ -10860,7 +10907,7 @@
       <c r="A179" s="9" t="s">
         <v>735</v>
       </c>
-      <c r="B179" s="17" t="s">
+      <c r="B179" s="14" t="s">
         <v>738</v>
       </c>
     </row>
@@ -10868,7 +10915,7 @@
       <c r="A180" s="4" t="s">
         <v>739</v>
       </c>
-      <c r="B180" s="17" t="s">
+      <c r="B180" s="14" t="s">
         <v>742</v>
       </c>
     </row>
@@ -10876,7 +10923,7 @@
       <c r="A181" s="9" t="s">
         <v>743</v>
       </c>
-      <c r="B181" s="17" t="s">
+      <c r="B181" s="14" t="s">
         <v>746</v>
       </c>
     </row>
@@ -10884,7 +10931,7 @@
       <c r="A182" s="4" t="s">
         <v>747</v>
       </c>
-      <c r="B182" s="17" t="s">
+      <c r="B182" s="14" t="s">
         <v>750</v>
       </c>
     </row>
@@ -10892,7 +10939,7 @@
       <c r="A183" s="9" t="s">
         <v>751</v>
       </c>
-      <c r="B183" s="17" t="s">
+      <c r="B183" s="14" t="s">
         <v>754</v>
       </c>
     </row>
@@ -10900,7 +10947,7 @@
       <c r="A184" s="4" t="s">
         <v>755</v>
       </c>
-      <c r="B184" s="17" t="s">
+      <c r="B184" s="14" t="s">
         <v>758</v>
       </c>
     </row>
@@ -10908,7 +10955,7 @@
       <c r="A185" s="9" t="s">
         <v>760</v>
       </c>
-      <c r="B185" s="17" t="s">
+      <c r="B185" s="14" t="s">
         <v>763</v>
       </c>
     </row>
@@ -10916,7 +10963,7 @@
       <c r="A186" s="4" t="s">
         <v>764</v>
       </c>
-      <c r="B186" s="17" t="s">
+      <c r="B186" s="14" t="s">
         <v>767</v>
       </c>
     </row>
@@ -10924,7 +10971,7 @@
       <c r="A187" s="9" t="s">
         <v>768</v>
       </c>
-      <c r="B187" s="17" t="s">
+      <c r="B187" s="14" t="s">
         <v>771</v>
       </c>
     </row>
@@ -10932,7 +10979,7 @@
       <c r="A188" s="4" t="s">
         <v>772</v>
       </c>
-      <c r="B188" s="17" t="s">
+      <c r="B188" s="14" t="s">
         <v>775</v>
       </c>
     </row>
@@ -10940,7 +10987,7 @@
       <c r="A189" s="9" t="s">
         <v>776</v>
       </c>
-      <c r="B189" s="17" t="s">
+      <c r="B189" s="14" t="s">
         <v>779</v>
       </c>
     </row>
@@ -10948,7 +10995,7 @@
       <c r="A190" s="4" t="s">
         <v>780</v>
       </c>
-      <c r="B190" s="17" t="s">
+      <c r="B190" s="14" t="s">
         <v>783</v>
       </c>
     </row>
@@ -10956,7 +11003,7 @@
       <c r="A191" s="9" t="s">
         <v>784</v>
       </c>
-      <c r="B191" s="17" t="s">
+      <c r="B191" s="14" t="s">
         <v>787</v>
       </c>
     </row>
@@ -10964,7 +11011,7 @@
       <c r="A192" s="4" t="s">
         <v>788</v>
       </c>
-      <c r="B192" s="17" t="s">
+      <c r="B192" s="14" t="s">
         <v>791</v>
       </c>
     </row>
@@ -10972,7 +11019,7 @@
       <c r="A193" s="9" t="s">
         <v>792</v>
       </c>
-      <c r="B193" s="17" t="s">
+      <c r="B193" s="14" t="s">
         <v>795</v>
       </c>
     </row>
@@ -10980,7 +11027,7 @@
       <c r="A194" s="4" t="s">
         <v>796</v>
       </c>
-      <c r="B194" s="17" t="s">
+      <c r="B194" s="14" t="s">
         <v>799</v>
       </c>
     </row>
@@ -10988,7 +11035,7 @@
       <c r="A195" s="9" t="s">
         <v>800</v>
       </c>
-      <c r="B195" s="17" t="s">
+      <c r="B195" s="14" t="s">
         <v>803</v>
       </c>
     </row>
@@ -10996,7 +11043,7 @@
       <c r="A196" s="4" t="s">
         <v>804</v>
       </c>
-      <c r="B196" s="17" t="s">
+      <c r="B196" s="14" t="s">
         <v>807</v>
       </c>
     </row>
@@ -11004,7 +11051,7 @@
       <c r="A197" s="9" t="s">
         <v>808</v>
       </c>
-      <c r="B197" s="17" t="s">
+      <c r="B197" s="14" t="s">
         <v>811</v>
       </c>
     </row>
@@ -11012,7 +11059,7 @@
       <c r="A198" s="4" t="s">
         <v>812</v>
       </c>
-      <c r="B198" s="17" t="s">
+      <c r="B198" s="14" t="s">
         <v>815</v>
       </c>
     </row>
@@ -11020,7 +11067,7 @@
       <c r="A199" s="9" t="s">
         <v>816</v>
       </c>
-      <c r="B199" s="17" t="s">
+      <c r="B199" s="14" t="s">
         <v>819</v>
       </c>
     </row>
@@ -11028,7 +11075,7 @@
       <c r="A200" s="4" t="s">
         <v>820</v>
       </c>
-      <c r="B200" s="17" t="s">
+      <c r="B200" s="14" t="s">
         <v>823</v>
       </c>
     </row>
@@ -11036,7 +11083,7 @@
       <c r="A201" s="9" t="s">
         <v>824</v>
       </c>
-      <c r="B201" s="17" t="s">
+      <c r="B201" s="14" t="s">
         <v>827</v>
       </c>
     </row>
@@ -11044,7 +11091,7 @@
       <c r="A202" s="4" t="s">
         <v>828</v>
       </c>
-      <c r="B202" s="17" t="s">
+      <c r="B202" s="14" t="s">
         <v>831</v>
       </c>
     </row>
@@ -11052,7 +11099,7 @@
       <c r="A203" s="9" t="s">
         <v>832</v>
       </c>
-      <c r="B203" s="17" t="s">
+      <c r="B203" s="14" t="s">
         <v>835</v>
       </c>
     </row>
@@ -11060,7 +11107,7 @@
       <c r="A204" s="4" t="s">
         <v>836</v>
       </c>
-      <c r="B204" s="17" t="s">
+      <c r="B204" s="14" t="s">
         <v>839</v>
       </c>
     </row>
@@ -11068,7 +11115,7 @@
       <c r="A205" s="9" t="s">
         <v>840</v>
       </c>
-      <c r="B205" s="17" t="s">
+      <c r="B205" s="14" t="s">
         <v>843</v>
       </c>
     </row>
@@ -11076,7 +11123,7 @@
       <c r="A206" s="4" t="s">
         <v>844</v>
       </c>
-      <c r="B206" s="17" t="s">
+      <c r="B206" s="14" t="s">
         <v>847</v>
       </c>
     </row>
@@ -11084,7 +11131,7 @@
       <c r="A207" s="9" t="s">
         <v>848</v>
       </c>
-      <c r="B207" s="17" t="s">
+      <c r="B207" s="14" t="s">
         <v>851</v>
       </c>
     </row>
@@ -11092,7 +11139,7 @@
       <c r="A208" s="4" t="s">
         <v>852</v>
       </c>
-      <c r="B208" s="17" t="s">
+      <c r="B208" s="14" t="s">
         <v>855</v>
       </c>
     </row>
@@ -11100,7 +11147,7 @@
       <c r="A209" s="9" t="s">
         <v>856</v>
       </c>
-      <c r="B209" s="17" t="s">
+      <c r="B209" s="14" t="s">
         <v>859</v>
       </c>
     </row>
@@ -11108,7 +11155,7 @@
       <c r="A210" s="4" t="s">
         <v>860</v>
       </c>
-      <c r="B210" s="17" t="s">
+      <c r="B210" s="14" t="s">
         <v>863</v>
       </c>
     </row>
@@ -11116,7 +11163,7 @@
       <c r="A211" s="9" t="s">
         <v>864</v>
       </c>
-      <c r="B211" s="17" t="s">
+      <c r="B211" s="14" t="s">
         <v>867</v>
       </c>
     </row>
@@ -11124,7 +11171,7 @@
       <c r="A212" s="4" t="s">
         <v>868</v>
       </c>
-      <c r="B212" s="17" t="s">
+      <c r="B212" s="14" t="s">
         <v>871</v>
       </c>
     </row>
@@ -11132,7 +11179,7 @@
       <c r="A213" s="9" t="s">
         <v>872</v>
       </c>
-      <c r="B213" s="17" t="s">
+      <c r="B213" s="14" t="s">
         <v>875</v>
       </c>
     </row>
@@ -11140,7 +11187,7 @@
       <c r="A214" s="4" t="s">
         <v>876</v>
       </c>
-      <c r="B214" s="17" t="s">
+      <c r="B214" s="14" t="s">
         <v>879</v>
       </c>
     </row>
@@ -11148,7 +11195,7 @@
       <c r="A215" s="9" t="s">
         <v>880</v>
       </c>
-      <c r="B215" s="17" t="s">
+      <c r="B215" s="14" t="s">
         <v>883</v>
       </c>
     </row>
@@ -11156,7 +11203,7 @@
       <c r="A216" s="4" t="s">
         <v>884</v>
       </c>
-      <c r="B216" s="17" t="s">
+      <c r="B216" s="14" t="s">
         <v>887</v>
       </c>
     </row>
@@ -11164,7 +11211,7 @@
       <c r="A217" s="9" t="s">
         <v>888</v>
       </c>
-      <c r="B217" s="17" t="s">
+      <c r="B217" s="14" t="s">
         <v>891</v>
       </c>
     </row>
@@ -11172,7 +11219,7 @@
       <c r="A218" s="4" t="s">
         <v>892</v>
       </c>
-      <c r="B218" s="17" t="s">
+      <c r="B218" s="14" t="s">
         <v>895</v>
       </c>
     </row>
@@ -11180,7 +11227,7 @@
       <c r="A219" s="9" t="s">
         <v>896</v>
       </c>
-      <c r="B219" s="17" t="s">
+      <c r="B219" s="14" t="s">
         <v>899</v>
       </c>
     </row>
@@ -11188,7 +11235,7 @@
       <c r="A220" s="4" t="s">
         <v>900</v>
       </c>
-      <c r="B220" s="17" t="s">
+      <c r="B220" s="14" t="s">
         <v>903</v>
       </c>
     </row>
@@ -11196,7 +11243,7 @@
       <c r="A221" s="9" t="s">
         <v>904</v>
       </c>
-      <c r="B221" s="17" t="s">
+      <c r="B221" s="14" t="s">
         <v>907</v>
       </c>
     </row>
@@ -11204,7 +11251,7 @@
       <c r="A222" s="4" t="s">
         <v>908</v>
       </c>
-      <c r="B222" s="17" t="s">
+      <c r="B222" s="14" t="s">
         <v>911</v>
       </c>
     </row>
@@ -11212,7 +11259,7 @@
       <c r="A223" s="9" t="s">
         <v>912</v>
       </c>
-      <c r="B223" s="17" t="s">
+      <c r="B223" s="14" t="s">
         <v>915</v>
       </c>
     </row>
@@ -11220,7 +11267,7 @@
       <c r="A224" s="4" t="s">
         <v>916</v>
       </c>
-      <c r="B224" s="17" t="s">
+      <c r="B224" s="14" t="s">
         <v>919</v>
       </c>
     </row>
@@ -11228,7 +11275,7 @@
       <c r="A225" s="9" t="s">
         <v>920</v>
       </c>
-      <c r="B225" s="17" t="s">
+      <c r="B225" s="14" t="s">
         <v>923</v>
       </c>
     </row>
@@ -11236,7 +11283,7 @@
       <c r="A226" s="4" t="s">
         <v>924</v>
       </c>
-      <c r="B226" s="17" t="s">
+      <c r="B226" s="14" t="s">
         <v>927</v>
       </c>
     </row>
@@ -11244,7 +11291,7 @@
       <c r="A227" s="9" t="s">
         <v>928</v>
       </c>
-      <c r="B227" s="17" t="s">
+      <c r="B227" s="14" t="s">
         <v>931</v>
       </c>
     </row>
@@ -11252,7 +11299,7 @@
       <c r="A228" s="4" t="s">
         <v>932</v>
       </c>
-      <c r="B228" s="17" t="s">
+      <c r="B228" s="14" t="s">
         <v>935</v>
       </c>
     </row>
@@ -11260,7 +11307,7 @@
       <c r="A229" s="9" t="s">
         <v>936</v>
       </c>
-      <c r="B229" s="17" t="s">
+      <c r="B229" s="14" t="s">
         <v>939</v>
       </c>
     </row>
@@ -11268,236 +11315,239 @@
       <c r="A230" s="4" t="s">
         <v>940</v>
       </c>
-      <c r="B230" s="17" t="s">
+      <c r="B230" s="14" t="s">
         <v>943</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A231" s="23" t="s">
+      <c r="A231" s="20" t="s">
         <v>961</v>
       </c>
-      <c r="B231" s="24" t="s">
+      <c r="B231" s="21" t="s">
         <v>964</v>
       </c>
     </row>
     <row r="232" spans="1:2" ht="15" x14ac:dyDescent="0.3">
-      <c r="A232" s="23" t="s">
+      <c r="A232" s="20" t="s">
         <v>1063</v>
       </c>
-      <c r="B232" s="24" t="s">
+      <c r="B232" s="21" t="s">
         <v>948</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A233" s="25" t="s">
+      <c r="A233" s="22" t="s">
         <v>949</v>
       </c>
-      <c r="B233" s="24" t="s">
+      <c r="B233" s="21" t="s">
         <v>952</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A234" s="23" t="s">
+      <c r="A234" s="20" t="s">
         <v>953</v>
       </c>
-      <c r="B234" s="24" t="s">
+      <c r="B234" s="21" t="s">
         <v>956</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A235" s="25" t="s">
+      <c r="A235" s="22" t="s">
         <v>957</v>
       </c>
-      <c r="B235" s="24" t="s">
+      <c r="B235" s="21" t="s">
         <v>960</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A236" s="25" t="s">
+      <c r="A236" s="22" t="s">
         <v>965</v>
       </c>
-      <c r="B236" s="24" t="s">
+      <c r="B236" s="21" t="s">
         <v>968</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A237" s="23" t="s">
+      <c r="A237" s="20" t="s">
         <v>969</v>
       </c>
-      <c r="B237" s="24" t="s">
+      <c r="B237" s="21" t="s">
         <v>972</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A238" s="25" t="s">
+      <c r="A238" s="22" t="s">
         <v>973</v>
       </c>
-      <c r="B238" s="24" t="s">
+      <c r="B238" s="21" t="s">
         <v>976</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A239" s="23" t="s">
+      <c r="A239" s="20" t="s">
         <v>977</v>
       </c>
-      <c r="B239" s="24" t="s">
+      <c r="B239" s="21" t="s">
         <v>980</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A240" s="25" t="s">
+      <c r="A240" s="22" t="s">
         <v>981</v>
       </c>
-      <c r="B240" s="24" t="s">
+      <c r="B240" s="21" t="s">
         <v>984</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A241" s="23" t="s">
+      <c r="A241" s="20" t="s">
         <v>985</v>
       </c>
-      <c r="B241" s="24" t="s">
+      <c r="B241" s="21" t="s">
         <v>988</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A242" s="25" t="s">
+      <c r="A242" s="22" t="s">
         <v>989</v>
       </c>
-      <c r="B242" s="24" t="s">
+      <c r="B242" s="21" t="s">
         <v>992</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A243" s="23" t="s">
+      <c r="A243" s="20" t="s">
         <v>993</v>
       </c>
-      <c r="B243" s="24" t="s">
+      <c r="B243" s="21" t="s">
         <v>996</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A244" s="25" t="s">
+      <c r="A244" s="22" t="s">
         <v>997</v>
       </c>
-      <c r="B244" s="24" t="s">
+      <c r="B244" s="21" t="s">
         <v>1000</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A245" s="23" t="s">
+      <c r="A245" s="20" t="s">
         <v>1001</v>
       </c>
-      <c r="B245" s="24" t="s">
+      <c r="B245" s="21" t="s">
         <v>1004</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A246" s="25" t="s">
+      <c r="A246" s="22" t="s">
         <v>1005</v>
       </c>
-      <c r="B246" s="24" t="s">
+      <c r="B246" s="21" t="s">
         <v>1008</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A247" s="23" t="s">
+      <c r="A247" s="20" t="s">
         <v>1009</v>
       </c>
-      <c r="B247" s="24" t="s">
+      <c r="B247" s="21" t="s">
         <v>1012</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A248" s="20" t="s">
+      <c r="A248" s="17" t="s">
         <v>1014</v>
       </c>
-      <c r="B248" s="21" t="s">
+      <c r="B248" s="18" t="s">
         <v>1017</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A249" s="22" t="s">
+      <c r="A249" s="19" t="s">
         <v>1018</v>
       </c>
-      <c r="B249" s="21" t="s">
+      <c r="B249" s="18" t="s">
         <v>1021</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A250" s="20" t="s">
+      <c r="A250" s="17" t="s">
         <v>1022</v>
       </c>
-      <c r="B250" s="21" t="s">
+      <c r="B250" s="18" t="s">
         <v>1025</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A251" s="22" t="s">
+      <c r="A251" s="19" t="s">
         <v>1026</v>
       </c>
-      <c r="B251" s="21" t="s">
+      <c r="B251" s="18" t="s">
         <v>1029</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A252" s="20" t="s">
+      <c r="A252" s="17" t="s">
         <v>1030</v>
       </c>
-      <c r="B252" s="21" t="s">
+      <c r="B252" s="18" t="s">
         <v>1033</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A253" s="22" t="s">
+      <c r="A253" s="19" t="s">
         <v>1034</v>
       </c>
-      <c r="B253" s="21" t="s">
+      <c r="B253" s="18" t="s">
         <v>1037</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A254" s="20" t="s">
+      <c r="A254" s="17" t="s">
         <v>1038</v>
       </c>
-      <c r="B254" s="21" t="s">
+      <c r="B254" s="18" t="s">
         <v>1041</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A255" s="22" t="s">
+      <c r="A255" s="19" t="s">
         <v>1042</v>
       </c>
-      <c r="B255" s="21" t="s">
+      <c r="B255" s="18" t="s">
         <v>1045</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A256" s="20" t="s">
+      <c r="A256" s="17" t="s">
         <v>1046</v>
       </c>
-      <c r="B256" s="21" t="s">
+      <c r="B256" s="18" t="s">
         <v>1049</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A257" s="22" t="s">
+      <c r="A257" s="19" t="s">
         <v>1050</v>
       </c>
-      <c r="B257" s="21" t="s">
+      <c r="B257" s="18" t="s">
         <v>1053</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A258" s="20" t="s">
+      <c r="A258" s="17" t="s">
         <v>1054</v>
       </c>
-      <c r="B258" s="21" t="s">
+      <c r="B258" s="18" t="s">
         <v>1057</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B59" r:id="rId1" xr:uid="{749BDCE0-BADC-4BF4-B324-07AC835B5943}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>